<commit_message>
Record live Timber audit verification
</commit_message>
<xml_diff>
--- a/Timber Course Alignment Audit.xlsx
+++ b/Timber Course Alignment Audit.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview &amp; Legend" sheetId="1" r:id="Rcf448a0dd26a4801"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Syllabus Alignment Matrix" sheetId="2" r:id="R3afeb0cd735b4976"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Evidence" sheetId="3" r:id="R9fa18db5c74d4843"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Register" sheetId="4" r:id="R7ccf8046f0a046cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gap Register" sheetId="5" r:id="R3ce27269267245d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Syllabus Summary" sheetId="6" r:id="Rd46bc5f6794a45e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Program Content Map" sheetId="7" r:id="Ra98e059dbceb4fbc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview &amp; Legend" sheetId="1" r:id="R3050c553c5ec4515"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Syllabus Alignment Matrix" sheetId="2" r:id="Rec065f48f56a4759"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Evidence" sheetId="3" r:id="Rcf2d1e2ccf0b4209"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Register" sheetId="4" r:id="R64472fad00504fd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gap Register" sheetId="5" r:id="R19c9f586a4854577"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Syllabus Summary" sheetId="6" r:id="R5501f87d503b454e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Program Content Map" sheetId="7" r:id="R21aa6e97873b4052"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -168,7 +168,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="34">
+  <x:fills count="35">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -328,6 +328,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFEAF2F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE6F0EB"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -646,7 +651,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="547">
+  <x:cellXfs count="552">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2096,6 +2101,21 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="24" fillId="33" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="14" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="15" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="34" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="34" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2538,7 +2558,7 @@
       <x:c r="G15" s="269"/>
       <x:c r="H15" s="269"/>
     </x:row>
-    <x:row r="16" ht="32" customHeight="1">
+    <x:row r="16" ht="112" customHeight="1">
       <x:c r="A16" s="265" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -2548,13 +2568,13 @@
       <x:c r="C16" s="276" t="str">
         <x:v>Year 9 · supplied current program</x:v>
       </x:c>
-      <x:c r="E16" s="507" t="str">
-        <x:f>"All ten current outcomes are addressed across the two-year pathway: "&amp;COUNTIF('Current Syllabus Summary'!B11:B20,"Covered")&amp;" Covered; "&amp;COUNTIF('Current Syllabus Summary'!B11:B20,"Partially covered")&amp;" Partially covered; "&amp;COUNTIF('Current Syllabus Summary'!B11:B20,"Has gaps")&amp;" Has gaps. IND56 is covered across the pathway; Mirror's local evidence repair awaits publication and live re-audit. IND59 is explicitly evidenced at Clock, with other full outcome lists clarified as course context. Of 77 unique current-program content statements, 75 occur in represented formal projects; two Pen-only lathe statements remain pending a course-sequence decision."</x:f>
-        <x:v>All ten current outcomes are addressed across the two-year pathway: 10 Covered; 0 Partially covered; 0 Has gaps. IND56 is covered across the pathway; Mirror's local evidence repair awaits publication and live re-audit. IND59 is explicitly evidenced at Clock, with other full outcome lists clarified as course context. Of 77 unique current-program content statements, 75 occur in represented formal projects; two Pen-only lathe statements remain pending a course-sequence decision.</x:v>
-      </x:c>
-      <x:c r="F16" s="507"/>
-      <x:c r="G16" s="507"/>
-      <x:c r="H16" s="507"/>
+      <x:c r="E16" s="547" t="str">
+        <x:f>"All ten current outcomes are addressed across the two-year pathway: "&amp;COUNTIF('Current Syllabus Summary'!B11:B20,"Covered")&amp;" Covered; "&amp;COUNTIF('Current Syllabus Summary'!B11:B20,"Partially covered")&amp;" Partially covered; "&amp;COUNTIF('Current Syllabus Summary'!B11:B20,"Has gaps")&amp;" Has gaps. IND56 now has live introductory, developed and evidenced collaboration records across Breadboard, Mirror and Bedside Table. IND59 is explicitly evidenced at Clock, with other project outcome lists verified as course context. No current outcome gap remains; the two Pen-only lathe content points remain an open program-scope decision."</x:f>
+        <x:v>All ten current outcomes are addressed across the two-year pathway: 10 Covered; 0 Partially covered; 0 Has gaps. IND56 now has live introductory, developed and evidenced collaboration records across Breadboard, Mirror and Bedside Table. IND59 is explicitly evidenced at Clock, with other project outcome lists verified as course context. No current outcome gap remains; the two Pen-only lathe content points remain an open program-scope decision.</x:v>
+      </x:c>
+      <x:c r="F16" s="547"/>
+      <x:c r="G16" s="547"/>
+      <x:c r="H16" s="547"/>
     </x:row>
     <x:row r="17" ht="32" customHeight="1">
       <x:c r="A17" s="292" t="n">
@@ -3207,7 +3227,7 @@
         <x:v>Weeks 9-10 drawing/CAD communication and Weeks 17-18 folio evidence.</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="66" customHeight="1">
+    <x:row r="12" ht="132" customHeight="1">
       <x:c r="A12" s="88" t="str">
         <x:v>Current program</x:v>
       </x:c>
@@ -3244,13 +3264,13 @@
       <x:c r="L12" s="113" t="str">
         <x:v>Weeks 15–16 team-lift and communication practice (CUR-01).</x:v>
       </x:c>
-      <x:c r="M12" s="522" t="str">
+      <x:c r="M12" s="548" t="str">
         <x:v>E</x:v>
       </x:c>
       <x:c r="N12" s="113" t="str">
-        <x:v>Local implementation 2026-08-02 - Mirror Portfolio Workbook, Peer Quality Check and Workshop Handover. Captures roles, criterion/evidence, feedback, justified decision, result check and handover contribution. Local QA complete; publication and live re-audit pending (S19).</x:v>
-      </x:c>
-      <x:c r="O12" s="493" t="str">
+        <x:v>Mirror Portfolio Workbook, Peer Quality Check and Workshop Handover - saved roles, criterion/evidence, feedback, justified decision, result check and handover contribution. Live verified 2026-08-02 at https://stevencowell.github.io/year-10-timber-mirror-project/mirror_portfolio_workbook.html (commit 9668c52; S19).</x:v>
+      </x:c>
+      <x:c r="O12" s="548" t="str">
         <x:v>E</x:v>
       </x:c>
       <x:c r="P12" s="113" t="str">
@@ -3375,7 +3395,7 @@
         <x:v>Weeks 17-18 criterion-based product evaluation and folio evidence.</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="66" customHeight="1">
+    <x:row r="15" ht="118" customHeight="1">
       <x:c r="A15" s="88" t="str">
         <x:v>Current program</x:v>
       </x:c>
@@ -3392,7 +3412,7 @@
         <x:v>Not applicable</x:v>
       </x:c>
       <x:c r="F15" s="113" t="str">
-        <x:v>Breadboard displays the course outcome list as context, not as a separate project-level IND59 assessment claim. Clock Weeks 15-16 remains the formal current-program E evidence for IND59; see Current Syllabus Summary IND59 and S19 local wording clarification.</x:v>
+        <x:v>Breadboard displays the course outcome list as context, not as a separate project-level IND59 assessment claim. Clock Weeks 15-16 remains the formal current-program E evidence for IND59. Course-context wording live verified 2026-08-02 (commit 11f7690; S19).</x:v>
       </x:c>
       <x:c r="G15" s="308" t="str">
         <x:v>Gap</x:v>
@@ -3412,17 +3432,17 @@
       <x:c r="L15" s="113" t="str">
         <x:v>Weeks 3-4 compares traditional and industrial timber production; no emerging-tech task.</x:v>
       </x:c>
-      <x:c r="M15" s="524" t="str">
+      <x:c r="M15" s="549" t="str">
         <x:v>Not applicable</x:v>
       </x:c>
       <x:c r="N15" s="113" t="str">
-        <x:v>Mirror displays the course outcome list as context, not as a separate project-level IND59 assessment claim. Clock Weeks 15-16 remains the formal current-program E evidence for IND59; see Current Syllabus Summary IND59 and S19 local wording clarification.</x:v>
-      </x:c>
-      <x:c r="O15" s="524" t="str">
+        <x:v>Mirror displays the course outcome list as context, not as a separate project-level IND59 assessment claim. Clock Weeks 15-16 remains the formal current-program E evidence for IND59. Course-context wording live verified 2026-08-02 (commit 9668c52; S19).</x:v>
+      </x:c>
+      <x:c r="O15" s="549" t="str">
         <x:v>Not applicable</x:v>
       </x:c>
       <x:c r="P15" s="113" t="str">
-        <x:v>Bedside Table displays the course outcome list as context, not as a separate project-level IND59 assessment claim. Clock Weeks 15-16 remains the formal current-program E evidence for IND59; see Current Syllabus Summary IND59 and S19 local wording clarification.</x:v>
+        <x:v>Bedside Table displays the course outcome list as context, not as a separate project-level IND59 assessment claim. Clock Weeks 15-16 remains the formal current-program E evidence for IND59. Course-context wording live verified 2026-08-02 (commit 9395842; S19).</x:v>
       </x:c>
       <x:c r="Q15" s="110" t="str">
         <x:v>E</x:v>
@@ -4191,7 +4211,7 @@
         <x:v>Date reviewed</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="142" customHeight="1">
+    <x:row r="5" ht="170" customHeight="1">
       <x:c r="A5" s="47" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -4212,10 +4232,10 @@
 Local implementation 2026-08-02 — Module 05 activity 1 captures peer feedback given/received, one improvement and a result check; it autosaves and is included in Print / Save PDF. Live verified 2026-08-02 (S18).</x:v>
       </x:c>
       <x:c r="G5" s="94" t="str">
-        <x:v>breadboard-folio.html is the selected public assessment-evidence destination: 12 project checkpoints, photo/caption evidence, autosave, backup and Print / Save PDF. It is not a formal task notification or marking rubric.</x:v>
+        <x:v>Live verified assessment-evidence destination: https://stevencowell.github.io/bread-board-guided-course/breadboard-folio.html - 12 project checkpoints, photo/caption evidence, autosave, backup and Print / Save PDF. It is not a formal task notification or marking rubric.</x:v>
       </x:c>
       <x:c r="H5" s="94" t="str">
-        <x:v>Assessment access decision recorded: use the project evidence folio. Formal task notices, dates, marks and Classroom submission remain teacher-controlled.</x:v>
+        <x:v>Assessment access closed and verified 2026-08-02. Formal task notices, dates, marks and Classroom submission remain teacher-controlled.</x:v>
       </x:c>
       <x:c r="I5" s="94" t="str">
         <x:v>Reviewed</x:v>
@@ -4297,7 +4317,7 @@
         <x:v>2026-08-01</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="92" customHeight="1">
+    <x:row r="8" ht="170" customHeight="1">
       <x:c r="A8" s="48" t="n">
         <x:v>4</x:v>
       </x:c>
@@ -4317,10 +4337,10 @@
         <x:v>10 guided modules with saved MCQ/written responses; printable Carry-all folio.</x:v>
       </x:c>
       <x:c r="G8" s="96" t="str">
-        <x:v>carry-all-folio.html is the selected public assessment-evidence destination: 12 project cards, responses/photos, progress, autosave, ZIP backup and Print / Save PDF. It is not a formal task notification or marking rubric.</x:v>
+        <x:v>Live verified assessment-evidence destination: https://stevencowell.github.io/Yr-9-Carry-All/carry-all-folio.html - 12 project cards, responses/photos, progress, autosave, ZIP backup and Print / Save PDF. It is not a formal task notification or marking rubric.</x:v>
       </x:c>
       <x:c r="H8" s="96" t="str">
-        <x:v>IND59 is introductory here. Assessment access decision recorded: use the project evidence folio; formal task notices and Classroom submission remain teacher-controlled.</x:v>
+        <x:v>IND59 is introductory here. Assessment access closed and verified 2026-08-02; formal task notices and Classroom submission remain teacher-controlled.</x:v>
       </x:c>
       <x:c r="I8" s="96" t="str">
         <x:v>Reviewed</x:v>
@@ -4332,7 +4352,7 @@
         <x:v>2026-08-01</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="92" customHeight="1">
+    <x:row r="9" ht="170" customHeight="1">
       <x:c r="A9" s="48" t="n">
         <x:v>5</x:v>
       </x:c>
@@ -4349,25 +4369,25 @@
         <x:v>Mirror-Project-Plans.pdf is linked from the live site.</x:v>
       </x:c>
       <x:c r="F9" s="96" t="str">
-        <x:v>9 live theory/activity pages, quizzes and editable portfolio workbook; separate folio; 20 repaired support-week routes. Local implementation 2026-08-02 - Portfolio Workbook Peer Quality Check and Workshop Handover captures a reviewer role, observable criterion/evidence, feedback, justified decision, result check and workshop handover; publication pending.</x:v>
+        <x:v>9 live theory/activity pages, quizzes and editable portfolio workbook; separate folio; 20 repaired support-week routes. The live Portfolio Workbook Peer Quality Check and Workshop Handover captures reviewer roles, observable criterion/evidence, feedback, a justified decision, result check and workshop handover.</x:v>
       </x:c>
       <x:c r="G9" s="96" t="str">
-        <x:v>mirror_assessment.html identifies practical, folio and class-test evidence. Local assessment-guide update adds the peer quality-check and handover record to portfolio evidence and rubric; publication pending.</x:v>
+        <x:v>mirror_assessment.html identifies practical, folio and class-test evidence and now includes the peer quality-check and handover record in the portfolio evidence checklist and rubric. Live verified 2026-08-02.</x:v>
       </x:c>
       <x:c r="H9" s="96" t="str">
-        <x:v>IND56 local repair awaits publication and live re-audit (CUR-01). IND59 is a course-context outcome here, not a separate Mirror evidence claim; Clock is the designated pathway E point (CUR-02).</x:v>
+        <x:v>IND56 project evidence is closed and verified. IND59 is course context here, not a separate Mirror assessment claim; Clock is the designated pathway E point.</x:v>
       </x:c>
       <x:c r="I9" s="96" t="str">
-        <x:v>Reviewed - local evidence repair pending publication</x:v>
+        <x:v>Reviewed - live evidence verified</x:v>
       </x:c>
       <x:c r="J9" s="33" t="str">
-        <x:v>Current-program project. Repaired support routes remain complete. Local collaboration record and assessment-rubric traceability were QA checked 2026-08-02; this does not assert individual student achievement.</x:v>
+        <x:v>Current-program project. Collaboration evidence and assessment-rubric traceability live verified 2026-08-02 (commit 9668c52; S19). This records an evidence opportunity, not individual student achievement.</x:v>
       </x:c>
       <x:c r="K9" s="34" t="str">
         <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="164" customHeight="1">
+    <x:row r="10" ht="170" customHeight="1">
       <x:c r="A10" s="48" t="n">
         <x:v>6</x:v>
       </x:c>
@@ -4388,10 +4408,10 @@
 Local implementation 2026-08-02 — Weeks 19–20 response 1 captures participant roles, peer QA critique, a justified technical decision, feedback-used evidence and workshop handover contribution; it autosaves and is included in Download PDF. Live verified 2026-08-02 (S18).</x:v>
       </x:c>
       <x:c r="G10" s="96" t="str">
-        <x:v>bedside-table-folio.html is the selected public assessment-evidence destination: 12 evidence cards, responses/photos, progress, ZIP/JSON backup and Print / Save PDF. It is not a formal task notification or marking rubric.</x:v>
+        <x:v>Live verified assessment-evidence destination: https://stevencowell.github.io/bedside-table-guided-course/bedside-table-folio.html - 12 evidence cards, responses/photos, progress, ZIP/JSON backup and Print / Save PDF. It is not a formal task notification or marking rubric.</x:v>
       </x:c>
       <x:c r="H10" s="96" t="str">
-        <x:v>Culminating evidence is broad. Assessment access decision recorded: use the project evidence folio; formal task notices and Classroom submission remain teacher-controlled. IND56 live evidence remains verified (S18).</x:v>
+        <x:v>Culminating evidence is broad. Assessment access closed and verified 2026-08-02; formal task notices and Classroom submission remain teacher-controlled. IND56 live evidence remains verified (S18).</x:v>
       </x:c>
       <x:c r="I10" s="96" t="str">
         <x:v>Reviewed</x:v>
@@ -5038,7 +5058,7 @@
         <x:v>Published and live verified 2026-08-02. Breadboard commit ad8c514: https://stevencowell.github.io/bread-board-guided-course/modules/module-05.html. Bedside Table commit 8fac5f5: https://stevencowell.github.io/bedside-table-guided-course/weeks19-20/. Both page activities were confirmed visible after GitHub Pages update.</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="120" customHeight="1">
+    <x:row r="23" ht="150" customHeight="1">
       <x:c r="A23" s="542" t="str">
         <x:v>S19</x:v>
       </x:c>
@@ -5058,10 +5078,10 @@
         <x:v>Mirror collaboration evidence; course-context clarification for IND59; verified Clock/Mirror assessment access; selected Breadboard, Carry-All and Bedside Table evidence-folio destinations; Pen trace note</x:v>
       </x:c>
       <x:c r="G23" s="543" t="str">
-        <x:v>Local QA complete 2026-08-02; publication and live re-audit pending</x:v>
+        <x:v>Published and live verified 2026-08-02</x:v>
       </x:c>
       <x:c r="H23" s="544" t="str">
-        <x:v>Selected folios: https://stevencowell.github.io/bread-board-guided-course/breadboard-folio.html; https://stevencowell.github.io/Yr-9-Carry-All/carry-all-folio.html; https://stevencowell.github.io/bedside-table-guided-course/bedside-table-folio.html. No unverified dates, marks, Classroom links or Pen project link were added.</x:v>
+        <x:v>Live verification: hub commit 82fe920; Breadboard 11f7690; Mirror 9668c52; Bedside Table 9395842; unchanged Carry-All folio at 31ff734. Verified routes: hub assessment section and workbook download; Breadboard, Carry-All and Bedside Table evidence folios; Clock assessment PDF; Mirror assessment guide and portfolio activity. No dates, marks, Classroom links or Pen project URL were invented.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5140,7 +5160,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="D6" s="367" t="str">
-        <x:v>CUR-01 and CUR-02 are locally repaired and await publication/live re-audit. CUR-03 remains an evidenced access issue for sites without a verified assessment destination. SCOPE-01 and SCOPE-02 are program-boundary decisions, not current outcome failures. Priority remains intentionally blank for Steve to set.</x:v>
+        <x:v>Current-program result: all ten outcomes are Covered across the two-year pathway and there are no open current-outcome gaps. CUR-01, CUR-02 and CUR-03 are retained below as closed, traceable repair records. SCOPE-01 and SCOPE-02 remain open program-boundary decisions, not current outcome failures. Priority ratings were not assigned by the audit and remain editable for Steve.</x:v>
       </x:c>
       <x:c r="E6" s="367"/>
       <x:c r="F6" s="367"/>
@@ -5208,67 +5228,67 @@
         <x:v>Status</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="116" customHeight="1">
+    <x:row r="12" ht="132" customHeight="1">
       <x:c r="A12" s="207" t="str"/>
       <x:c r="B12" s="213" t="str">
         <x:v>Mirror</x:v>
       </x:c>
       <x:c r="C12" s="193" t="str">
-        <x:v>CUR-01 - Mirror now has a local peer quality-check and workshop-handover evidence record; publication and live re-audit remain required.</x:v>
+        <x:v>CUR-01 - closed action: Mirror collaboration evidence is published and live verified.</x:v>
       </x:c>
       <x:c r="D12" s="193" t="str">
-        <x:v>The IND56 record now captures roles, observable criterion/evidence, feedback, a justified technical decision, feedback used and a shared-workshop handover. This extends the existing Year 9-to-Year 10 scaffold without claiming individual achievement.</x:v>
+        <x:v>The record captures roles, an observable criterion, feedback, a justified technical decision, evidence of feedback used and workshop handover. It adds a visible Year 10 evidence point without claiming individual achievement.</x:v>
       </x:c>
       <x:c r="E12" s="193" t="str">
-        <x:v>Local Mirror Portfolio Workbook and mirror_assessment.html update, 2026-08-02; Matrix row 12; Project Evidence row 9; Source Register S19.</x:v>
+        <x:v>https://stevencowell.github.io/year-10-timber-mirror-project/mirror_portfolio_workbook.html; mirror_assessment.html; commit 9668c52; Matrix row 12; Project Evidence row 9; S19; verified 2026-08-02.</x:v>
       </x:c>
       <x:c r="F12" s="193" t="str">
-        <x:v>Commit and publish the three local Mirror files, then confirm the live workbook activity and assessment-guide criterion before closing.</x:v>
-      </x:c>
-      <x:c r="G12" s="528" t="str">
-        <x:v>Resolved - re-audit required</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="94" customHeight="1">
+        <x:v>Use the activity during delivery and sample student portfolio/PDF evidence through normal faculty assessment processes.</x:v>
+      </x:c>
+      <x:c r="G12" s="550" t="str">
+        <x:v>Closed - verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="132" customHeight="1">
       <x:c r="A13" s="208" t="str"/>
       <x:c r="B13" s="214" t="str">
         <x:v>Breadboard; Clock; Tool Carry-all; Mirror; Bedside Table</x:v>
       </x:c>
       <x:c r="C13" s="196" t="str">
-        <x:v>CUR-02 - IND59 evidence is now clearly sequenced: Clock is the formal current-program E point; Carry-all is an introductory comparison; full outcome lists on Breadboard, Mirror and Bedside Table are course context only.</x:v>
+        <x:v>CUR-02 - closed action: IND59 evidence is explicitly sequenced and broad outcome-list claims are clarified.</x:v>
       </x:c>
       <x:c r="D13" s="196" t="str">
-        <x:v>This prevents a reviewer treating every project outcome list as a separate assessment claim. The two-year pathway retains one explicit formal evidence point rather than generic duplicated commentary.</x:v>
+        <x:v>Clock remains the formal current-program E point; Carry-All introduces the comparison; Breadboard, Mirror and Bedside Table now identify their outcome lists as course context rather than separate assessment claims.</x:v>
       </x:c>
       <x:c r="E13" s="196" t="str">
-        <x:v>Current Syllabus Summary IND59; Matrix row 15; local course-context wording updates at Breadboard, Mirror and Bedside Table; Source Register S19.</x:v>
+        <x:v>Current Syllabus Summary IND59; Matrix row 15; live landing pages; Breadboard 11f7690, Mirror 9668c52, Bedside Table 9395842; S19; verified 2026-08-02.</x:v>
       </x:c>
       <x:c r="F13" s="196" t="str">
-        <x:v>Commit and publish the local wording updates, then live recheck the three landing pages. No additional generic technology activity is required for pathway coverage.</x:v>
-      </x:c>
-      <x:c r="G13" s="534" t="str">
-        <x:v>Resolved - re-audit required</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="122" customHeight="1">
+        <x:v>Retain Clock as the explicit IND59 evidence point unless the formal program is revised. No duplicated generic technology activity is required.</x:v>
+      </x:c>
+      <x:c r="G13" s="551" t="str">
+        <x:v>Closed - verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="132" customHeight="1">
       <x:c r="A14" s="208" t="str"/>
       <x:c r="B14" s="214" t="str">
         <x:v>Breadboard; Tool Carry-all; Bedside Table</x:v>
       </x:c>
       <x:c r="C14" s="196" t="str">
-        <x:v>CUR-03 - project-specific assessment-evidence destinations have been selected and added to the local hub; publication and live verification remain required.</x:v>
+        <x:v>CUR-03 - closed action: the hub now links each project's strongest verified assessment-evidence folio.</x:v>
       </x:c>
       <x:c r="D14" s="196" t="str">
-        <x:v>Each repository has a strong editable student evidence folio but no separate public task notification or marking rubric. The hub labels them as evidence folios so a reviewer can open the strongest real destination without overclaiming what it is.</x:v>
+        <x:v>These are editable student evidence folios, not formal task notifications or marking rubrics. The distinction keeps assessment access useful without inventing school-controlled details.</x:v>
       </x:c>
       <x:c r="E14" s="196" t="str">
-        <x:v>Bread Board Project Folio: https://stevencowell.github.io/bread-board-guided-course/breadboard-folio.html; Carry-All Student Project Folio: https://stevencowell.github.io/Yr-9-Carry-All/carry-all-folio.html; Bedside Table Student Folio: https://stevencowell.github.io/bedside-table-guided-course/bedside-table-folio.html; Source Register S19.</x:v>
+        <x:v>Breadboard: https://stevencowell.github.io/bread-board-guided-course/breadboard-folio.html; Carry-All: https://stevencowell.github.io/Yr-9-Carry-All/carry-all-folio.html; Bedside Table: https://stevencowell.github.io/bedside-table-guided-course/bedside-table-folio.html; hub commit 82fe920; verified 2026-08-02.</x:v>
       </x:c>
       <x:c r="F14" s="196" t="str">
-        <x:v>Publish the hub link update, then verify all three folio routes and labels live. Keep task notices, dates, marks and Classroom links teacher-controlled unless a verified destination is later supplied.</x:v>
-      </x:c>
-      <x:c r="G14" s="546" t="str">
-        <x:v>Resolved - re-audit required</x:v>
+        <x:v>Keep dates, marks, task notices and Classroom destinations teacher-controlled unless verified faculty sources are later supplied.</x:v>
+      </x:c>
+      <x:c r="G14" s="551" t="str">
+        <x:v>Closed - verified</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="94" customHeight="1">
@@ -5610,7 +5630,7 @@
         <x:v>Retain the named folio, drawing, caption, portfolio and PDF outputs as the communication trail.</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="116" customHeight="1">
+    <x:row r="16" ht="148" customHeight="1">
       <x:c r="A16" s="266" t="str">
         <x:v>IND56</x:v>
       </x:c>
@@ -5622,13 +5642,13 @@
         <x:v>identifies and participates in collaborative work practices in the learning environment</x:v>
       </x:c>
       <x:c r="D16" s="196" t="str">
-        <x:v>Stage 1 Breadboard introduces a structured peer-feedback record. The Mirror Portfolio Workbook now adds a local Year 10 peer quality check: named roles, criterion/evidence, feedback, a justified decision, result check and workshop handover. Bedside Table retains the deeper live peer QA response. The record deepens across Years 9-10; Mirror publication and live re-audit remain pending.</x:v>
+        <x:v>Stage 1 Breadboard introduces structured peer feedback and one recorded improvement. Stage 5 Mirror evidences a criterion-based peer quality check, a justified technical decision and workshop handover. Stage 6 Bedside Table deepens this through peer QA, before/after evidence and named handover roles. The evidence opportunity progresses from introduced to practised and evidenced across Years 9-10.</x:v>
       </x:c>
       <x:c r="E16" s="196" t="str">
-        <x:v>Matrix row 12; Breadboard Module 05 live activity; Mirror Portfolio Workbook local Peer Quality Check and Workshop Handover; Bedside Table Weeks 19-20 live response; Project Evidence rows 5, 9 and 10; Source Register S18-S19.</x:v>
+        <x:v>Matrix row 12; Breadboard Module 05; Mirror Portfolio Workbook Peer Quality Check and Workshop Handover; Bedside Table Weeks 19-20; Project Evidence rows 5, 9 and 10; Source Register S18-S19. All three live records verified 2026-08-02.</x:v>
       </x:c>
       <x:c r="F16" s="197" t="str">
-        <x:v>Pathway evidence is covered. Mirror's project-level evidence is locally repaired and awaits publication/live re-audit; individual student achievement is not asserted.</x:v>
+        <x:v>Pathway and Mirror project evidence are live and verified. Continue sampling actual student folio/PDF evidence during delivery; this audit does not assert individual achievement.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="96" customHeight="1">
@@ -5673,7 +5693,7 @@
         <x:v>Retain the criterion-linked Year 10 evaluation and reflection evidence.</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="96" customHeight="1">
+    <x:row r="19" ht="126" customHeight="1">
       <x:c r="A19" s="266" t="str">
         <x:v>IND59</x:v>
       </x:c>
@@ -5685,13 +5705,13 @@
         <x:v>describes, analyses and uses a range of current, new and emerging technologies and their various applications</x:v>
       </x:c>
       <x:c r="D19" s="196" t="str">
-        <x:v>Clock Weeks 15-16 is the explicit formal-current evidence point. Carry-all provides a later introductory comparison; Breadboard, Mirror and Bedside Table list the outcome for course context but do not claim a separate project-level IND59 assessment.</x:v>
+        <x:v>Clock Weeks 15-16 is the explicit formal-current evidence point. Carry-All provides an introductory comparison. Breadboard, Mirror and Bedside Table display the outcome list as course context and do not claim separate project-level IND59 assessment.</x:v>
       </x:c>
       <x:c r="E19" s="196" t="str">
-        <x:v>Matrix row 15; Clock Weeks 15-16; Carry-all Weeks 3-4; local course-context wording updates recorded at S19.</x:v>
+        <x:v>Matrix row 15; Clock Weeks 15-16; Carry-All Weeks 3-4; live Breadboard, Mirror and Bedside Table course-context wording; Source Register S19; verified 2026-08-02.</x:v>
       </x:c>
       <x:c r="F19" s="197" t="str">
-        <x:v>Pathway coverage is retained through Clock. Local wording clarification awaits publication/live re-audit; no generic duplicated technology activity is required.</x:v>
+        <x:v>Pathway coverage is retained through Clock. The course-context clarification is live; no duplicated generic technology activity is required.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="96" customHeight="1">

</xml_diff>

<commit_message>
Record Pen program decision in Timber audit
</commit_message>
<xml_diff>
--- a/Timber Course Alignment Audit.xlsx
+++ b/Timber Course Alignment Audit.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview &amp; Legend" sheetId="1" r:id="R3050c553c5ec4515"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Syllabus Alignment Matrix" sheetId="2" r:id="Rec065f48f56a4759"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Evidence" sheetId="3" r:id="Rcf2d1e2ccf0b4209"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Register" sheetId="4" r:id="R64472fad00504fd2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gap Register" sheetId="5" r:id="R19c9f586a4854577"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Syllabus Summary" sheetId="6" r:id="R5501f87d503b454e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Program Content Map" sheetId="7" r:id="R21aa6e97873b4052"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview &amp; Legend" sheetId="1" r:id="Re3a8fd16f9a74cb2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Syllabus Alignment Matrix" sheetId="2" r:id="R422721ea9b9e41ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Evidence" sheetId="3" r:id="R1c6fd3f5def94ece"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Register" sheetId="4" r:id="R2e94d81ebd3d4a7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gap Register" sheetId="5" r:id="Re90acb56b6974310"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Syllabus Summary" sheetId="6" r:id="R82c4e6d433794f41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Program Content Map" sheetId="7" r:id="R53ecccc08ef44c6c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -168,7 +168,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="35">
+  <x:fills count="39">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -338,6 +338,26 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFE6F0EB"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE6F0EB"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF3F5F4"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -651,7 +671,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="552">
+  <x:cellXfs count="570">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2117,6 +2137,60 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="24" fillId="34" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="8" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="8" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="36" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="36" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="36" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="37" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="37" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="37" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="37" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="38" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="36" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="38" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="36" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -2558,7 +2632,7 @@
       <x:c r="G15" s="269"/>
       <x:c r="H15" s="269"/>
     </x:row>
-    <x:row r="16" ht="112" customHeight="1">
+    <x:row r="16" ht="132" customHeight="1">
       <x:c r="A16" s="265" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -2569,8 +2643,8 @@
         <x:v>Year 9 · supplied current program</x:v>
       </x:c>
       <x:c r="E16" s="547" t="str">
-        <x:f>"All ten current outcomes are addressed across the two-year pathway: "&amp;COUNTIF('Current Syllabus Summary'!B11:B20,"Covered")&amp;" Covered; "&amp;COUNTIF('Current Syllabus Summary'!B11:B20,"Partially covered")&amp;" Partially covered; "&amp;COUNTIF('Current Syllabus Summary'!B11:B20,"Has gaps")&amp;" Has gaps. IND56 now has live introductory, developed and evidenced collaboration records across Breadboard, Mirror and Bedside Table. IND59 is explicitly evidenced at Clock, with other project outcome lists verified as course context. No current outcome gap remains; the two Pen-only lathe content points remain an open program-scope decision."</x:f>
-        <x:v>All ten current outcomes are addressed across the two-year pathway: 10 Covered; 0 Partially covered; 0 Has gaps. IND56 now has live introductory, developed and evidenced collaboration records across Breadboard, Mirror and Bedside Table. IND59 is explicitly evidenced at Clock, with other project outcome lists verified as course context. No current outcome gap remains; the two Pen-only lathe content points remain an open program-scope decision.</x:v>
+        <x:f>"All ten current outcomes are addressed across the two-year pathway: "&amp;COUNTIF('Current Syllabus Summary'!B11:B20,"Covered")&amp;" Covered; "&amp;COUNTIF('Current Syllabus Summary'!B11:B20,"Partially covered")&amp;" Partially covered; "&amp;COUNTIF('Current Syllabus Summary'!B11:B20,"Has gaps")&amp;" Has gaps. Current-program content map: "&amp;COUNTIF('Current Program Content Map'!H16:H92,"Mapped")&amp;" of "&amp;COUNTA('Current Program Content Map'!A16:A92)&amp;" statements mapped; "&amp;COUNTIF('Current Program Content Map'!H16:H92,"Has gaps")&amp;" gaps. Pen is retained as an unnumbered Year 9 woodturning mini-unit, normally after Clock and before Tool Carry-all; the source also permits delivery after Carry-all. The seven hub stages remain unchanged."</x:f>
+        <x:v>All ten current outcomes are addressed across the two-year pathway: 10 Covered; 0 Partially covered; 0 Has gaps. Current-program content map: 77 of 77 statements mapped; 0 gaps. Pen is retained as an unnumbered Year 9 woodturning mini-unit, normally after Clock and before Tool Carry-all; the source also permits delivery after Carry-all. The seven hub stages remain unchanged.</x:v>
       </x:c>
       <x:c r="F16" s="547"/>
       <x:c r="G16" s="547"/>
@@ -4143,7 +4217,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="7" t="str">
-        <x:v>Reviewed evidence register in the required teaching sequence. Findings describe what the published site can teach or capture; they do not substitute for teacher observation, submitted student work or an authorised assessment schedule.</x:v>
+        <x:v>Reviewed evidence register for the seven numbered hub projects. Pen is recorded below as an unnumbered current-program mini-unit so its evidence remains auditable without changing the agreed hub scaffold. Findings describe what the published site can teach or capture; they do not substitute for teacher observation, submitted student work or an authorised assessment schedule.</x:v>
       </x:c>
       <x:c r="B3" s="7" t="str">
         <x:v>Reviewed evidence register in the required teaching sequence. Findings describe what the published site can teach or capture; they do not substitute for teacher observation, submitted student work or an authorised assessment schedule.</x:v>
@@ -4456,6 +4530,41 @@
       </x:c>
       <x:c r="K11" s="343" t="str">
         <x:v>2026-08-01</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="210" customHeight="1">
+      <x:c r="A12" s="555" t="str">
+        <x:v>Embedded</x:v>
+      </x:c>
+      <x:c r="B12" s="553" t="str">
+        <x:v>Pen</x:v>
+      </x:c>
+      <x:c r="C12" s="553" t="str">
+        <x:v>Year 9 · supplied current program; unnumbered woodturning mini-unit</x:v>
+      </x:c>
+      <x:c r="D12" s="553" t="str">
+        <x:v>https://stevencowell.github.io/Yr-9-Pen/</x:v>
+      </x:c>
+      <x:c r="E12" s="553" t="str">
+        <x:v>Approved Pen Making process resource linked from the current site: https://docs.google.com/presentation/d/1u0JvcPVGXRjNzHRATh9hTASWldvNeBqBCgvCW9pY4I8/edit</x:v>
+      </x:c>
+      <x:c r="F12" s="553" t="str">
+        <x:v>Selected core evidence: Weeks 3–4 timber selection and grain response; Weeks 5–6 blank/sleeve preparation; Weeks 7–8 supervised mandrel setup and pre-start check; Weeks 9–10 controlled turning; Weeks 11–12 surface and finish checks. Written responses autosave and can be printed/saved as PDF.</x:v>
+      </x:c>
+      <x:c r="G12" s="553" t="str">
+        <x:v>Student folio: https://stevencowell.github.io/Yr-9-Pen/pen-folio.html — cards 4–9 record timber selection, preparation, supervised setup, controlled turning, surface diagnosis and finishing. The editable local Pen assessment/evidence plan adds teacher-observation checkpoints: C:\Users\scowell1\Documents\Codex\2026-07-29\realtime-voice-chat-3\outputs\pen-teacher-pack\pen-assessment-evidence-plan.docx</x:v>
+      </x:c>
+      <x:c r="H12" s="553" t="str">
+        <x:v>No unresolved current-content gap. The source contains a genuine duration inconsistency (one week, two weekly rows, and a one-to-two-week overview). The 20-week guided-site structure is an evidence/support bank, not the formal mini-unit duration. Actual delivery and student achievement remain locally verified.</x:v>
+      </x:c>
+      <x:c r="I12" s="553" t="str">
+        <x:v>Reviewed - course decision recorded</x:v>
+      </x:c>
+      <x:c r="J12" s="553" t="str">
+        <x:v>Decision 2026-08-02: retain Pen. Plan a two-week practical mini-unit by default, preferably after Clock and before Tool Carry-all; the source permits delivery after Carry-all. Pen remains outside the seven numbered hub stages.</x:v>
+      </x:c>
+      <x:c r="K12" s="553" t="str">
+        <x:v>2026-08-02</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5084,6 +5193,32 @@
         <x:v>Live verification: hub commit 82fe920; Breadboard 11f7690; Mirror 9668c52; Bedside Table 9395842; unchanged Carry-All folio at 31ff734. Verified routes: hub assessment section and workbook download; Breadboard, Carry-All and Bedside Table evidence folios; Clock assessment PDF; Mirror assessment guide and portfolio activity. No dates, marks, Classroom links or Pen project URL were invented.</x:v>
       </x:c>
     </x:row>
+    <x:row r="24" ht="190" customHeight="1">
+      <x:c r="A24" s="555" t="str">
+        <x:v>S20</x:v>
+      </x:c>
+      <x:c r="B24" s="553" t="str">
+        <x:v>Pen current-program decision and evidence map</x:v>
+      </x:c>
+      <x:c r="C24" s="553" t="str">
+        <x:v>Current course decision / verified guided-course evidence</x:v>
+      </x:c>
+      <x:c r="D24" s="553" t="str">
+        <x:v>Year 9 embedded woodturning unit; CP038 and CP039</x:v>
+      </x:c>
+      <x:c r="E24" s="553" t="str">
+        <x:v>Primary program: C:\Users\scowell1\Downloads\stage_5_timber_2021-06-16.docx, tables 22–24. Current guided course: https://stevencowell.github.io/Yr-9-Pen/. Approved Pen Making process resource: https://docs.google.com/presentation/d/1u0JvcPVGXRjNzHRATh9hTASWldvNeBqBCgvCW9pY4I8/edit. Local planning aid: C:\Users\scowell1\Documents\Codex\2026-07-29\realtime-voice-chat-3\outputs\pen-teacher-pack\pen-assessment-evidence-plan.docx</x:v>
+      </x:c>
+      <x:c r="F24" s="553" t="str">
+        <x:v>Program sequence and unit role; timber-selection/preparation responses; supervised setup and between-centres turning activities; dedicated folio cards 4–9; teacher-observation checkpoints.</x:v>
+      </x:c>
+      <x:c r="G24" s="553" t="str">
+        <x:v>Decision recorded; live evidence verified 2026-08-02</x:v>
+      </x:c>
+      <x:c r="H24" s="553" t="str">
+        <x:v>Retain Pen as an unnumbered Year 9 mini-unit. Use the source's complete two-row sequence as the default two-week plan; preferred placement is after Clock and before Tool Carry-all, while the source permits delivery after Carry-all. The current 20-week Pen site is an evidence/support bank and does not redefine formal duration. Yr-9-Pen main verified at commit 6fe4c7f. The local teacher pack is a planning aid, not source authority or proof of delivery.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
@@ -5160,7 +5295,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="D6" s="367" t="str">
-        <x:v>Current-program result: all ten outcomes are Covered across the two-year pathway and there are no open current-outcome gaps. CUR-01, CUR-02 and CUR-03 are retained below as closed, traceable repair records. SCOPE-01 and SCOPE-02 remain open program-boundary decisions, not current outcome failures. Priority ratings were not assigned by the audit and remain editable for Steve.</x:v>
+        <x:v>Current-program result: all ten outcomes are Covered across the two-year pathway and all 77 exact current-program content statements are mapped. CUR-01, CUR-02, CUR-03 and SCOPE-01 are retained below as closed, traceable records. SCOPE-02 remains an open program-boundary label for local additions, not a current-outcome or current-content failure. Priority ratings were not assigned by the audit and remain editable for Steve.</x:v>
       </x:c>
       <x:c r="E6" s="367"/>
       <x:c r="F6" s="367"/>
@@ -5291,25 +5426,25 @@
         <x:v>Closed - verified</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="94" customHeight="1">
-      <x:c r="A15" s="208" t="str"/>
+    <x:row r="15" ht="170" customHeight="1">
+      <x:c r="A15" s="205" t="str"/>
       <x:c r="B15" s="214" t="str">
         <x:v>Pen</x:v>
       </x:c>
       <x:c r="C15" s="196" t="str">
-        <x:v>SCOPE-01 - Pen is now visibly traced on the local hub and audit, but its formal placement, duration and two lathe-specific content points still need a course decision and evidence location.</x:v>
+        <x:v>SCOPE-01 - closed course decision: Pen is retained as an unnumbered Year 9 woodturning mini-unit, with explicit evidence locations for CP038 and CP039.</x:v>
       </x:c>
       <x:c r="D15" s="196" t="str">
-        <x:v>The current program names Pen, while the agreed hub pathway does not include it. The local audit makes the boundary visible without claiming that 77/77 content points are represented.</x:v>
+        <x:v>This restores traceability for the two Pen-only lathe statements without forcing Pen into the seven numbered hub stages. The source is internally inconsistent about one versus two weeks, so the complete two-row sequence is the safer default planning baseline.</x:v>
       </x:c>
       <x:c r="E15" s="196" t="str">
-        <x:v>Current Program Content Map CP038 and CP039; current program tables 21-24; local hub program-trace note.</x:v>
+        <x:v>Current program tables 22–24; Project Evidence row 12; Current Program Content Map CP038–CP039; https://stevencowell.github.io/Yr-9-Pen/ modules Weeks 3–12; https://stevencowell.github.io/Yr-9-Pen/pen-folio.html cards 4–9; S20; live verified 2026-08-02.</x:v>
       </x:c>
       <x:c r="F15" s="196" t="str">
-        <x:v>Steve to confirm whether Pen is retained, omitted or replaced, and which duration governs. Then map the two content points or formally record the replacement.</x:v>
-      </x:c>
-      <x:c r="G15" s="535" t="str">
-        <x:v>Open - course decision needed</x:v>
+        <x:v>Deliver the selected timber-preparation, supervised setup and controlled-turning evidence within the local program. Use two weeks by default; if local timing compresses delivery or moves it after Carry-all, record that timetable decision. Sample actual student folio and teacher-observation evidence during delivery.</x:v>
+      </x:c>
+      <x:c r="G15" s="560" t="str">
+        <x:v>Closed - verified</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="94" customHeight="1">
@@ -5467,7 +5602,7 @@
       <x:c r="E6" s="227"/>
       <x:c r="F6" s="227"/>
     </x:row>
-    <x:row r="7">
+    <x:row r="7" ht="82" customHeight="1">
       <x:c r="A7" s="404" t="str">
         <x:v>Covered</x:v>
       </x:c>
@@ -5475,13 +5610,13 @@
         <x:f>COUNTIF($B$11:$B$20,A7)</x:f>
         <x:v>10</x:v>
       </x:c>
-      <x:c r="D7" s="412" t="str">
-        <x:v>Supplied current-program sequence: Breadboard → Clock → Pen (additional turning unit after Clock or Carry-all) → Tool Carry-all → Mirror → Bedside Table. The Pen duration is inconsistent in the source (1 week, 2-week sequence and 1–2 week overview). Audited hub sequence: Breadboard → Small Box (local) → Clock → Tool Carry-all → Mirror → Bedside Table → Folding Chair (local developing option). Pen lacks an audited hub trace; local additions are excluded from the formal-current status calculation.</x:v>
-      </x:c>
-      <x:c r="E7" s="412"/>
-      <x:c r="F7" s="412"/>
-    </x:row>
-    <x:row r="8">
+      <x:c r="D7" s="561" t="str">
+        <x:v>Supplied current-program sequence for this companion: Breadboard → Clock → Pen (embedded Year 9 woodturning mini-unit) → Tool Carry-all → Mirror → Bedside Table. Decision 2026-08-02: retain Pen, plan the complete two-row sequence as two weeks by default, and place it after Clock and before Tool Carry-all where practical; the source also permits delivery after Carry-all. The seven numbered hub stages remain unchanged. The current Pen guided course and folio provide auditable evidence opportunities; their 20-week navigation does not redefine the short formal unit.</x:v>
+      </x:c>
+      <x:c r="E7" s="561"/>
+      <x:c r="F7" s="561"/>
+    </x:row>
+    <x:row r="8" ht="82" customHeight="1">
       <x:c r="A8" s="406" t="str">
         <x:v>Partially covered</x:v>
       </x:c>
@@ -5489,11 +5624,11 @@
         <x:f>COUNTIF($B$11:$B$20,A8)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D8" s="412"/>
-      <x:c r="E8" s="412"/>
-      <x:c r="F8" s="412"/>
-    </x:row>
-    <x:row r="9">
+      <x:c r="D8" s="561"/>
+      <x:c r="E8" s="561"/>
+      <x:c r="F8" s="561"/>
+    </x:row>
+    <x:row r="9" ht="82" customHeight="1">
       <x:c r="A9" s="408" t="str">
         <x:v>Has gaps</x:v>
       </x:c>
@@ -5501,9 +5636,9 @@
         <x:f>COUNTIF($B$11:$B$20,A9)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D9" s="412"/>
-      <x:c r="E9" s="412"/>
-      <x:c r="F9" s="412"/>
+      <x:c r="D9" s="561"/>
+      <x:c r="E9" s="561"/>
+      <x:c r="F9" s="561"/>
     </x:row>
     <x:row r="10" ht="36" customHeight="1">
       <x:c r="A10" s="370" t="str">
@@ -5567,7 +5702,7 @@
         <x:v>Keep the later approved design decisions as the evidence point that completes Breadboard practice.</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="96" customHeight="1">
+    <x:row r="13" ht="118" customHeight="1">
       <x:c r="A13" s="266" t="str">
         <x:v>IND53</x:v>
       </x:c>
@@ -5579,16 +5714,16 @@
         <x:v>identifies, selects and uses a range of hand and machine tools, equipment and processes to produce quality practical projects</x:v>
       </x:c>
       <x:c r="D13" s="196" t="str">
-        <x:v>Breadboard basic marking and jointing → Clock and Carry-all multi-step production → Mirror and Bedside Table complex joinery, jigs, assembly and finishing.</x:v>
+        <x:v>Breadboard basic marking and jointing → Clock and Carry-all multi-step production → embedded Pen supervised mandrel setup and controlled turning → Mirror and Bedside Table complex joinery, jigs, assembly and finishing.</x:v>
       </x:c>
       <x:c r="E13" s="196" t="str">
-        <x:v>Matrix row 9; Breadboard Modules 02–04; Clock Weeks 5–14; Carry-all Weeks 5–18; Mirror process activities; Bedside Table Weeks 3–16.</x:v>
+        <x:v>Matrix row 9; Breadboard Modules 02–04; Clock Weeks 5–14; Carry-all Weeks 5–18; Pen Weeks 7–12 and folio cards 6–9 (Project Evidence row 12; S20); Mirror process activities; Bedside Table Weeks 3–16.</x:v>
       </x:c>
       <x:c r="F13" s="197" t="str">
-        <x:v>Retain the nominated production records across simple, multi-step and complex joinery stages.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="96" customHeight="1">
+        <x:v>Retain the nominated production records across basic, multi-step, supervised turning and complex joinery stages.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="118" customHeight="1">
       <x:c r="A14" s="266" t="str">
         <x:v>IND54</x:v>
       </x:c>
@@ -5600,13 +5735,13 @@
         <x:v>selects, justifies and uses a range of relevant and associated materials for specific applications</x:v>
       </x:c>
       <x:c r="D14" s="196" t="str">
-        <x:v>Breadboard grain/layout selection → Clock and Carry-all timber choice and responsible use → Year 10 cutting lists, matched grain and application-specific selection.</x:v>
+        <x:v>Breadboard grain/layout selection → Clock and Carry-all timber choice and responsible use → embedded Pen blank inspection, grain orientation and preparation → Year 10 cutting lists, matched grain and application-specific selection.</x:v>
       </x:c>
       <x:c r="E14" s="196" t="str">
-        <x:v>Matrix row 10; Breadboard Module 02; Clock Weeks 3–4 and 11–12; Carry-all Weeks 3–4; Mirror materials/cutting list; Bedside Table Weeks 3–4.</x:v>
+        <x:v>Matrix row 10; Breadboard Module 02; Clock Weeks 3–4 and 11–12; Carry-all Weeks 3–4; Pen Weeks 3–6 and folio cards 4–5 (Project Evidence row 12; S20); Mirror materials/cutting list; Bedside Table Weeks 3–4.</x:v>
       </x:c>
       <x:c r="F14" s="197" t="str">
-        <x:v>Retain the project-specific timber selection and justification records across the sequence.</x:v>
+        <x:v>Retain the Pen timber-selection record and the project-specific material justifications across the sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="96" customHeight="1">
@@ -5651,7 +5786,7 @@
         <x:v>Pathway and Mirror project evidence are live and verified. Continue sampling actual student folio/PDF evidence during delivery; this audit does not assert individual achievement.</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="96" customHeight="1">
+    <x:row r="17" ht="118" customHeight="1">
       <x:c r="A17" s="266" t="str">
         <x:v>IND57</x:v>
       </x:c>
@@ -5663,16 +5798,16 @@
         <x:v>applies and transfers skills, processes and materials to a variety of contexts and projects</x:v>
       </x:c>
       <x:c r="D17" s="196" t="str">
-        <x:v>Breadboard transfer remains implicit → Clock, Carry-all and Bedside Table require explicit future-use or problem-solving transfer evidence; Mirror remains practised/developed.</x:v>
+        <x:v>Breadboard transfer remains implicit → Clock and Carry-all require explicit transfer evidence → embedded Pen transfers timber reading, marking and safe-machine habits into turning → Mirror remains developed and Bedside Table evidences future-use/problem-solving transfer.</x:v>
       </x:c>
       <x:c r="E17" s="196" t="str">
-        <x:v>Matrix row 13; Clock and Bedside Table Weeks 19–20; Carry-all Weeks 5–6 and 19–20; Breadboard/Mirror supporting practice.</x:v>
+        <x:v>Matrix row 13; Clock and Bedside Table Weeks 19–20; Carry-all Weeks 5–6 and 19–20; Pen course and final folio card 12 (Project Evidence row 12; S20); Breadboard/Mirror supporting practice.</x:v>
       </x:c>
       <x:c r="F17" s="197" t="str">
-        <x:v>Retain the later explicit transfer prompts that complete the earlier implicit practice.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="96" customHeight="1">
+        <x:v>Retain the later explicit transfer prompts and Pen final reflection that complete the earlier practice.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="118" customHeight="1">
       <x:c r="A18" s="266" t="str">
         <x:v>IND58</x:v>
       </x:c>
@@ -5684,13 +5819,13 @@
         <x:v>evaluates products in terms of functional, economic, aesthetic and environmental qualities and quality of construction</x:v>
       </x:c>
       <x:c r="D18" s="196" t="str">
-        <x:v>Early PMI/folio evaluation → Carry-all problem-correction evidence → Year 10 criterion-based product evaluation and final reflection.</x:v>
+        <x:v>Early PMI/folio evaluation → Carry-all problem-correction evidence → embedded Pen surface, finish and final-quality judgements → Year 10 criterion-based product evaluation and final reflection.</x:v>
       </x:c>
       <x:c r="E18" s="196" t="str">
-        <x:v>Matrix row 14; folio/PMI evaluation at Breadboard and Clock; problem correction at Carry-all; criterion-based Year 10 evaluation.</x:v>
+        <x:v>Matrix row 14; folio/PMI evaluation at Breadboard and Clock; problem correction at Carry-all; Pen Weeks 11–12 and folio cards 8–12 (Project Evidence row 12; S20); criterion-based Year 10 evaluation.</x:v>
       </x:c>
       <x:c r="F18" s="197" t="str">
-        <x:v>Retain the criterion-linked Year 10 evaluation and reflection evidence.</x:v>
+        <x:v>Retain the Pen surface/finish evidence and criterion-linked Year 10 evaluation trail.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="126" customHeight="1">
@@ -5851,10 +5986,10 @@
       </x:c>
       <x:c r="F7" s="405" t="n">
         <x:f>COUNTIF($H$16:$H$92,E7)</x:f>
-        <x:v>75</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="H7" s="412" t="str">
-        <x:v>Mapped means the exact statement occurs in at least one formal project represented in the audited hub. It does not claim an exact webpage module match unless a page is named elsewhere. Has gaps is reserved for the two Pen-only lathe statements: the program contains them, but no Pen project/site evidence row exists. Named teaching activities, student evidence and resources are preserved from the source rather than inferred.</x:v>
+        <x:v>Mapped means the exact statement occurs in the supplied current program and has a named program placement. Where a verified site activity or folio exists, its location is identified in the row. All 77 statements are now mapped; CP038 and CP039 use the retained Pen mini-unit, current Pen guided-course activities and folio evidence. This records an available evidence pathway, not proof of lesson delivery, individual student achievement, departmental approval or a dot-point-to-IND crosswalk.</x:v>
       </x:c>
       <x:c r="I7" s="412"/>
       <x:c r="J7" s="412"/>
@@ -5874,7 +6009,7 @@
       </x:c>
       <x:c r="F8" s="409" t="n">
         <x:f>COUNTIF($H$16:$H$92,E8)</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H8" s="412"/>
       <x:c r="I8" s="412"/>
@@ -7702,75 +7837,75 @@
       </x:c>
     </x:row>
     <x:row r="53" ht="75.5999984741211" hidden="0" customHeight="1">
-      <x:c r="A53" s="477" t="str">
+      <x:c r="A53" s="568" t="str">
         <x:v>CP038</x:v>
       </x:c>
-      <x:c r="B53" s="478" t="str">
+      <x:c r="B53" s="563" t="str">
         <x:v>select and prepare timber for the lathe, for example:</x:v>
       </x:c>
-      <x:c r="C53" s="478" t="str">
+      <x:c r="C53" s="563" t="str">
         <x:v>between centres turning</x:v>
       </x:c>
-      <x:c r="D53" s="478" t="str">
+      <x:c r="D53" s="563" t="str">
         <x:v>Pen Week 1
 Pen Week 2</x:v>
       </x:c>
-      <x:c r="E53" s="478" t="str">
+      <x:c r="E53" s="563" t="str">
         <x:v>Pen Week 1: Demonstration of turning. Practice on scrap.
 Pen Week 2: Work on and complete pen.</x:v>
       </x:c>
-      <x:c r="F53" s="478" t="str">
+      <x:c r="F53" s="563" t="str">
         <x:v>Pen Week 1: Theory: Discussion: Types of uses for the Wood Lathe Workbook/Folio: Risk management for using the Lathe Practical: Demonstrate / Observe: Setup and demonstrate turning techniques. Simple scraping and cutting between centres Sanding and finishing on the lathe Turn a timber pen - Start to finish | Resource: No resource location stated in source row.
 Pen Week 2: Demonstrate / Observe: Setup for turning. Simple scraping and cutting between centres - Techniques Sanding and finishing on the lathe Turn a timber pen - Start to finish | Resource: No resource location stated in source row.</x:v>
       </x:c>
-      <x:c r="G53" s="478" t="str">
-        <x:v>Pen: SCOPE-01; no Project Evidence row</x:v>
-      </x:c>
-      <x:c r="H53" s="479" t="str">
-        <x:v>Has gaps</x:v>
-      </x:c>
-      <x:c r="I53" s="478" t="str">
+      <x:c r="G53" s="563" t="str">
+        <x:v>Pen embedded unit: Project Evidence row 12; https://stevencowell.github.io/Yr-9-Pen/weeks3-4/ (timber selection and grain response); https://stevencowell.github.io/Yr-9-Pen/weeks5-6/ (blank/sleeve preparation); https://stevencowell.github.io/Yr-9-Pen/pen-folio.html cards 4–5; S20.</x:v>
+      </x:c>
+      <x:c r="H53" s="569" t="str">
+        <x:v>Mapped</x:v>
+      </x:c>
+      <x:c r="I53" s="563" t="str">
         <x:v>stage_5_timber_2021-06-16.docx, table 24, row 1
 stage_5_timber_2021-06-16.docx, table 24, row 2</x:v>
       </x:c>
-      <x:c r="J53" s="480" t="str">
-        <x:v>SCOPE-01 — confirm Pen is retained and evidenced, or formally map a replacement.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="54" ht="75.5999984741211" hidden="0" customHeight="1">
-      <x:c r="A54" s="477" t="str">
+      <x:c r="J53" s="565" t="str">
+        <x:v>Decision 2026-08-02: retained as a short Year 9 woodturning unit. Plan the source's complete two-row sequence as two weeks by default; selected Pen pages and folio cards provide the inspectable timber-selection/preparation evidence opportunity. The source permits placement after Clock or Carry-all.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="118.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A54" s="568" t="str">
         <x:v>CP039</x:v>
       </x:c>
-      <x:c r="B54" s="478" t="str">
+      <x:c r="B54" s="563" t="str">
         <x:v>set up and use lathe techniques for basic turning processes, for example:</x:v>
       </x:c>
-      <x:c r="C54" s="478" t="str">
+      <x:c r="C54" s="563" t="str">
         <x:v>between centres turning, eg rolling pin, mallet handle</x:v>
       </x:c>
-      <x:c r="D54" s="478" t="str">
+      <x:c r="D54" s="563" t="str">
         <x:v>Pen Week 1
 Pen Week 2</x:v>
       </x:c>
-      <x:c r="E54" s="478" t="str">
+      <x:c r="E54" s="563" t="str">
         <x:v>Pen Week 1: Demonstration of turning. Practice on scrap.
 Pen Week 2: Work on and complete pen.</x:v>
       </x:c>
-      <x:c r="F54" s="478" t="str">
+      <x:c r="F54" s="563" t="str">
         <x:v>Pen Week 1: Theory: Discussion: Types of uses for the Wood Lathe Workbook/Folio: Risk management for using the Lathe Practical: Demonstrate / Observe: Setup and demonstrate turning techniques. Simple scraping and cutting between centres Sanding and finishing on the lathe Turn a timber pen - Start to finish | Resource: No resource location stated in source row.
 Pen Week 2: Demonstrate / Observe: Setup for turning. Simple scraping and cutting between centres - Techniques Sanding and finishing on the lathe Turn a timber pen - Start to finish | Resource: No resource location stated in source row.</x:v>
       </x:c>
-      <x:c r="G54" s="478" t="str">
-        <x:v>Pen: SCOPE-01; no Project Evidence row</x:v>
-      </x:c>
-      <x:c r="H54" s="479" t="str">
-        <x:v>Has gaps</x:v>
-      </x:c>
-      <x:c r="I54" s="478" t="str">
+      <x:c r="G54" s="563" t="str">
+        <x:v>Pen embedded unit: Project Evidence row 12; https://stevencowell.github.io/Yr-9-Pen/weeks7-8/ (between-centres principles, mandrel and pre-start); https://stevencowell.github.io/Yr-9-Pen/weeks9-10/ (controlled cutting/scraping and profile development); https://stevencowell.github.io/Yr-9-Pen/weeks11-12/ (surface/finish checks); https://stevencowell.github.io/Yr-9-Pen/pen-folio.html cards 6–9; S20.</x:v>
+      </x:c>
+      <x:c r="H54" s="569" t="str">
+        <x:v>Mapped</x:v>
+      </x:c>
+      <x:c r="I54" s="563" t="str">
         <x:v>stage_5_timber_2021-06-16.docx, table 24, row 1
 stage_5_timber_2021-06-16.docx, table 24, row 2</x:v>
       </x:c>
-      <x:c r="J54" s="480" t="str">
-        <x:v>SCOPE-01 — confirm Pen is retained and evidenced, or formally map a replacement.</x:v>
+      <x:c r="J54" s="565" t="str">
+        <x:v>Decision 2026-08-02: mapped to supervised setup, approved workholding, controlled turning and finishing evidence. Teacher approval, local SOPs and observation remain required; the mapping is an evidence opportunity, not proof of individual achievement.</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="43.20000076293945" hidden="0" customHeight="1">

</xml_diff>